<commit_message>
new project 29 and 30
</commit_message>
<xml_diff>
--- a/Project_Roadmap_Ashwini.xlsx
+++ b/Project_Roadmap_Ashwini.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\E drive\Previous data\Project\52 project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E5FADB-323F-43D3-9904-48F2E7357855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECCF7044-7CF5-4645-9CF5-421718D4A68E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9050,6 +9050,7 @@
       </c>
     </row>
     <row r="32" spans="1:12">
+      <c r="A32" s="6"/>
       <c r="B32" s="1">
         <v>27</v>
       </c>
@@ -9085,7 +9086,8 @@
         <v>232</v>
       </c>
     </row>
-    <row r="33" spans="2:12">
+    <row r="33" spans="1:12">
+      <c r="A33" s="6"/>
       <c r="B33" s="1">
         <v>28</v>
       </c>
@@ -9121,7 +9123,8 @@
         <v>235</v>
       </c>
     </row>
-    <row r="34" spans="2:12">
+    <row r="34" spans="1:12">
+      <c r="A34" s="6"/>
       <c r="B34" s="1">
         <v>29</v>
       </c>
@@ -9157,7 +9160,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="35" spans="2:12">
+    <row r="35" spans="1:12">
       <c r="B35" s="1">
         <v>30</v>
       </c>
@@ -9193,7 +9196,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="36" spans="2:12">
+    <row r="36" spans="1:12">
       <c r="B36" s="1">
         <v>31</v>
       </c>
@@ -9229,7 +9232,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="37" spans="2:12" ht="27.6">
+    <row r="37" spans="1:12" ht="27.6">
       <c r="B37" s="1">
         <v>32</v>
       </c>
@@ -9265,7 +9268,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="38" spans="2:12" ht="27.6">
+    <row r="38" spans="1:12" ht="27.6">
       <c r="B38" s="1">
         <v>33</v>
       </c>
@@ -9301,7 +9304,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="39" spans="2:12">
+    <row r="39" spans="1:12">
       <c r="B39" s="1">
         <v>34</v>
       </c>
@@ -9337,7 +9340,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="40" spans="2:12">
+    <row r="40" spans="1:12">
       <c r="B40" s="1">
         <v>35</v>
       </c>
@@ -9373,7 +9376,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="41" spans="2:12">
+    <row r="41" spans="1:12">
       <c r="B41" s="1">
         <v>36</v>
       </c>
@@ -9409,7 +9412,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="42" spans="2:12" ht="27.6">
+    <row r="42" spans="1:12" ht="27.6">
       <c r="B42" s="1">
         <v>37</v>
       </c>
@@ -9445,7 +9448,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="43" spans="2:12" ht="27.6">
+    <row r="43" spans="1:12" ht="27.6">
       <c r="B43" s="1">
         <v>38</v>
       </c>
@@ -9481,7 +9484,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="44" spans="2:12">
+    <row r="44" spans="1:12">
       <c r="B44" s="1">
         <v>39</v>
       </c>
@@ -9517,7 +9520,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="45" spans="2:12">
+    <row r="45" spans="1:12">
       <c r="B45" s="1">
         <v>40</v>
       </c>
@@ -9553,7 +9556,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="46" spans="2:12">
+    <row r="46" spans="1:12">
       <c r="B46" s="1">
         <v>41</v>
       </c>
@@ -9589,7 +9592,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="47" spans="2:12">
+    <row r="47" spans="1:12">
       <c r="B47" s="1">
         <v>42</v>
       </c>
@@ -9625,7 +9628,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="48" spans="2:12" ht="27.6">
+    <row r="48" spans="1:12" ht="27.6">
       <c r="B48" s="1">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
Added new project folders (46-75) and updated roadmap
Excluded real .env secrets and an oversized .rar (>100MB GitHub limit)
via .gitignore; two empty scaffold repos (YouTube StoryForge Agent,
Neural-Semantic Matching Protocol) left untracked for now.
</commit_message>
<xml_diff>
--- a/Project_Roadmap_Ashwini.xlsx
+++ b/Project_Roadmap_Ashwini.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\E drive\Previous data\Project\52 project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4C82B8-65E9-4FDD-A377-759092D16229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9FEE16F-199D-41B7-84F8-4D498051A1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -1388,7 +1388,7 @@
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1428,8 +1428,13 @@
       <color rgb="FF7F6000"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1472,6 +1477,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1485,7 +1496,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1518,6 +1529,8 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9420,6 +9433,7 @@
       </c>
     </row>
     <row r="42" spans="1:12" ht="27.6">
+      <c r="A42" s="6"/>
       <c r="B42" s="1">
         <v>37</v>
       </c>
@@ -9456,6 +9470,7 @@
       </c>
     </row>
     <row r="43" spans="1:12" ht="27.6">
+      <c r="A43" s="6"/>
       <c r="B43" s="1">
         <v>38</v>
       </c>
@@ -9528,6 +9543,7 @@
       </c>
     </row>
     <row r="45" spans="1:12">
+      <c r="A45" s="6"/>
       <c r="B45" s="1">
         <v>40</v>
       </c>
@@ -9564,6 +9580,7 @@
       </c>
     </row>
     <row r="46" spans="1:12">
+      <c r="A46" s="6"/>
       <c r="B46" s="1">
         <v>41</v>
       </c>
@@ -9600,6 +9617,7 @@
       </c>
     </row>
     <row r="47" spans="1:12">
+      <c r="A47" s="6"/>
       <c r="B47" s="1">
         <v>42</v>
       </c>
@@ -9636,6 +9654,7 @@
       </c>
     </row>
     <row r="48" spans="1:12" ht="27.6">
+      <c r="A48" s="6"/>
       <c r="B48" s="1">
         <v>43</v>
       </c>
@@ -9671,7 +9690,8 @@
         <v>269</v>
       </c>
     </row>
-    <row r="49" spans="2:12" ht="27.6">
+    <row r="49" spans="1:12" ht="27.6">
+      <c r="A49" s="6"/>
       <c r="B49" s="1">
         <v>44</v>
       </c>
@@ -9707,7 +9727,8 @@
         <v>270</v>
       </c>
     </row>
-    <row r="50" spans="2:12">
+    <row r="50" spans="1:12">
+      <c r="A50" s="6"/>
       <c r="B50" s="1">
         <v>45</v>
       </c>
@@ -9743,7 +9764,8 @@
         <v>273</v>
       </c>
     </row>
-    <row r="51" spans="2:12">
+    <row r="51" spans="1:12">
+      <c r="A51" s="6"/>
       <c r="B51" s="1">
         <v>46</v>
       </c>
@@ -9779,7 +9801,8 @@
         <v>274</v>
       </c>
     </row>
-    <row r="52" spans="2:12" ht="27.6">
+    <row r="52" spans="1:12" ht="27.6">
+      <c r="A52" s="6"/>
       <c r="B52" s="1">
         <v>47</v>
       </c>
@@ -9815,7 +9838,8 @@
         <v>277</v>
       </c>
     </row>
-    <row r="53" spans="2:12">
+    <row r="53" spans="1:12">
+      <c r="A53" s="6"/>
       <c r="B53" s="1">
         <v>48</v>
       </c>
@@ -9851,7 +9875,8 @@
         <v>280</v>
       </c>
     </row>
-    <row r="54" spans="2:12">
+    <row r="54" spans="1:12">
+      <c r="A54" s="6"/>
       <c r="B54" s="1">
         <v>49</v>
       </c>
@@ -9887,7 +9912,8 @@
         <v>283</v>
       </c>
     </row>
-    <row r="55" spans="2:12" ht="27.6">
+    <row r="55" spans="1:12" ht="27.6">
+      <c r="A55" s="6"/>
       <c r="B55" s="1">
         <v>50</v>
       </c>
@@ -9923,7 +9949,8 @@
         <v>286</v>
       </c>
     </row>
-    <row r="56" spans="2:12" ht="27.6">
+    <row r="56" spans="1:12" ht="27.6">
+      <c r="A56" s="6"/>
       <c r="B56" s="1">
         <v>51</v>
       </c>
@@ -9959,7 +9986,8 @@
         <v>289</v>
       </c>
     </row>
-    <row r="57" spans="2:12" ht="27.6">
+    <row r="57" spans="1:12" ht="27.6">
+      <c r="A57" s="6"/>
       <c r="B57" s="1">
         <v>52</v>
       </c>
@@ -9995,7 +10023,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="58" spans="2:12">
+    <row r="58" spans="1:12">
       <c r="B58" s="1">
         <v>53</v>
       </c>
@@ -10031,7 +10059,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="59" spans="2:12">
+    <row r="59" spans="1:12">
       <c r="B59" s="1">
         <v>54</v>
       </c>
@@ -10067,7 +10095,8 @@
         <v>296</v>
       </c>
     </row>
-    <row r="60" spans="2:12" ht="27.6">
+    <row r="60" spans="1:12" ht="27.6">
+      <c r="A60" s="6"/>
       <c r="B60" s="1">
         <v>55</v>
       </c>
@@ -10103,7 +10132,8 @@
         <v>299</v>
       </c>
     </row>
-    <row r="61" spans="2:12">
+    <row r="61" spans="1:12">
+      <c r="A61" s="6"/>
       <c r="B61" s="1">
         <v>56</v>
       </c>
@@ -10139,7 +10169,8 @@
         <v>302</v>
       </c>
     </row>
-    <row r="62" spans="2:12">
+    <row r="62" spans="1:12">
+      <c r="A62" s="6"/>
       <c r="B62" s="1">
         <v>57</v>
       </c>
@@ -10175,7 +10206,8 @@
         <v>303</v>
       </c>
     </row>
-    <row r="63" spans="2:12" ht="27.6">
+    <row r="63" spans="1:12" ht="27.6">
+      <c r="A63" s="6"/>
       <c r="B63" s="1">
         <v>58</v>
       </c>
@@ -10211,7 +10243,10 @@
         <v>306</v>
       </c>
     </row>
-    <row r="64" spans="2:12">
+    <row r="64" spans="1:12">
+      <c r="A64" s="6">
+        <v>29</v>
+      </c>
       <c r="B64" s="1">
         <v>59</v>
       </c>
@@ -10247,7 +10282,8 @@
         <v>309</v>
       </c>
     </row>
-    <row r="65" spans="2:12" ht="27.6">
+    <row r="65" spans="1:12" ht="27.6">
+      <c r="A65" s="6"/>
       <c r="B65" s="1">
         <v>60</v>
       </c>
@@ -10283,7 +10319,8 @@
         <v>310</v>
       </c>
     </row>
-    <row r="66" spans="2:12">
+    <row r="66" spans="1:12">
+      <c r="A66" s="6"/>
       <c r="B66" s="1">
         <v>61</v>
       </c>
@@ -10319,7 +10356,8 @@
         <v>311</v>
       </c>
     </row>
-    <row r="67" spans="2:12" ht="27.6">
+    <row r="67" spans="1:12" ht="27.6">
+      <c r="A67" s="6"/>
       <c r="B67" s="1">
         <v>62</v>
       </c>
@@ -10355,7 +10393,8 @@
         <v>313</v>
       </c>
     </row>
-    <row r="68" spans="2:12">
+    <row r="68" spans="1:12">
+      <c r="A68" s="6"/>
       <c r="B68" s="1">
         <v>63</v>
       </c>
@@ -10391,7 +10430,10 @@
         <v>314</v>
       </c>
     </row>
-    <row r="69" spans="2:12" ht="27.6">
+    <row r="69" spans="1:12" ht="27.6">
+      <c r="A69" s="6">
+        <v>30</v>
+      </c>
       <c r="B69" s="1">
         <v>64</v>
       </c>
@@ -10427,7 +10469,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="70" spans="2:12" ht="27.6">
+    <row r="70" spans="1:12" ht="27.6">
       <c r="B70" s="1">
         <v>65</v>
       </c>
@@ -10463,7 +10505,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="71" spans="2:12" ht="27.6">
+    <row r="71" spans="1:12" ht="27.6">
       <c r="B71" s="1">
         <v>66</v>
       </c>
@@ -10499,7 +10541,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="72" spans="2:12">
+    <row r="72" spans="1:12">
       <c r="B72" s="1">
         <v>67</v>
       </c>
@@ -10535,7 +10577,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="73" spans="2:12" ht="27.6">
+    <row r="73" spans="1:12" ht="27.6">
       <c r="B73" s="1">
         <v>68</v>
       </c>
@@ -10571,7 +10613,10 @@
         <v>326</v>
       </c>
     </row>
-    <row r="74" spans="2:12" ht="27.6">
+    <row r="74" spans="1:12" ht="27.6">
+      <c r="A74" s="6">
+        <v>31</v>
+      </c>
       <c r="B74" s="1">
         <v>69</v>
       </c>
@@ -10607,7 +10652,8 @@
         <v>328</v>
       </c>
     </row>
-    <row r="75" spans="2:12">
+    <row r="75" spans="1:12">
+      <c r="A75" s="6"/>
       <c r="B75" s="1">
         <v>70</v>
       </c>
@@ -10643,7 +10689,8 @@
         <v>331</v>
       </c>
     </row>
-    <row r="76" spans="2:12">
+    <row r="76" spans="1:12">
+      <c r="A76" s="12"/>
       <c r="B76" s="1">
         <v>71</v>
       </c>
@@ -10679,7 +10726,8 @@
         <v>334</v>
       </c>
     </row>
-    <row r="77" spans="2:12" ht="27.6">
+    <row r="77" spans="1:12" ht="27.6">
+      <c r="A77" s="6"/>
       <c r="B77" s="1">
         <v>72</v>
       </c>
@@ -10715,7 +10763,8 @@
         <v>335</v>
       </c>
     </row>
-    <row r="78" spans="2:12" ht="27.6">
+    <row r="78" spans="1:12" ht="27.6">
+      <c r="A78" s="13"/>
       <c r="B78" s="1">
         <v>73</v>
       </c>
@@ -10751,7 +10800,10 @@
         <v>338</v>
       </c>
     </row>
-    <row r="79" spans="2:12" ht="27.6">
+    <row r="79" spans="1:12" ht="27.6">
+      <c r="A79">
+        <v>1</v>
+      </c>
       <c r="B79" s="1">
         <v>74</v>
       </c>
@@ -10787,7 +10839,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="80" spans="2:12">
+    <row r="80" spans="1:12">
       <c r="B80" s="1">
         <v>75</v>
       </c>
@@ -10823,7 +10875,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="81" spans="2:12" ht="27.6">
+    <row r="81" spans="1:12" ht="27.6">
       <c r="B81" s="1">
         <v>76</v>
       </c>
@@ -10859,7 +10911,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="82" spans="2:12">
+    <row r="82" spans="1:12">
       <c r="B82" s="1">
         <v>77</v>
       </c>
@@ -10895,7 +10947,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="83" spans="2:12" ht="27.6">
+    <row r="83" spans="1:12" ht="27.6">
       <c r="B83" s="1">
         <v>78</v>
       </c>
@@ -10931,7 +10983,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="84" spans="2:12" ht="27.6">
+    <row r="84" spans="1:12" ht="27.6">
+      <c r="A84">
+        <v>2</v>
+      </c>
       <c r="B84" s="1">
         <v>79</v>
       </c>
@@ -10967,7 +11022,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="85" spans="2:12" ht="27.6">
+    <row r="85" spans="1:12" ht="27.6">
       <c r="B85" s="1">
         <v>80</v>
       </c>
@@ -11003,7 +11058,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="86" spans="2:12">
+    <row r="86" spans="1:12">
       <c r="B86" s="4"/>
       <c r="C86" s="4"/>
       <c r="D86" s="4"/>
@@ -11016,7 +11071,7 @@
       <c r="K86" s="4"/>
       <c r="L86" s="4"/>
     </row>
-    <row r="87" spans="2:12">
+    <row r="87" spans="1:12">
       <c r="B87" s="4"/>
       <c r="C87" s="4"/>
       <c r="D87" s="4"/>
@@ -11029,7 +11084,7 @@
       <c r="K87" s="4"/>
       <c r="L87" s="4"/>
     </row>
-    <row r="88" spans="2:12">
+    <row r="88" spans="1:12">
       <c r="B88" s="4"/>
       <c r="C88" s="4"/>
       <c r="D88" s="4"/>
@@ -11042,7 +11097,7 @@
       <c r="K88" s="4"/>
       <c r="L88" s="4"/>
     </row>
-    <row r="89" spans="2:12">
+    <row r="89" spans="1:12">
       <c r="B89" s="4"/>
       <c r="C89" s="4"/>
       <c r="D89" s="4"/>
@@ -11055,7 +11110,7 @@
       <c r="K89" s="4"/>
       <c r="L89" s="4"/>
     </row>
-    <row r="90" spans="2:12">
+    <row r="90" spans="1:12">
       <c r="B90" s="4"/>
       <c r="C90" s="4"/>
       <c r="D90" s="4"/>
@@ -11068,7 +11123,7 @@
       <c r="K90" s="4"/>
       <c r="L90" s="4"/>
     </row>
-    <row r="91" spans="2:12">
+    <row r="91" spans="1:12">
       <c r="B91" s="4"/>
       <c r="C91" s="4"/>
       <c r="D91" s="4"/>
@@ -11081,7 +11136,7 @@
       <c r="K91" s="4"/>
       <c r="L91" s="4"/>
     </row>
-    <row r="92" spans="2:12">
+    <row r="92" spans="1:12">
       <c r="B92" s="4"/>
       <c r="C92" s="4"/>
       <c r="D92" s="4"/>
@@ -11094,7 +11149,7 @@
       <c r="K92" s="4"/>
       <c r="L92" s="4"/>
     </row>
-    <row r="93" spans="2:12">
+    <row r="93" spans="1:12">
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
       <c r="D93" s="4"/>
@@ -11107,7 +11162,7 @@
       <c r="K93" s="4"/>
       <c r="L93" s="4"/>
     </row>
-    <row r="94" spans="2:12">
+    <row r="94" spans="1:12">
       <c r="B94" s="4"/>
       <c r="C94" s="4"/>
       <c r="D94" s="4"/>
@@ -11120,7 +11175,7 @@
       <c r="K94" s="4"/>
       <c r="L94" s="4"/>
     </row>
-    <row r="95" spans="2:12">
+    <row r="95" spans="1:12">
       <c r="B95" s="4"/>
       <c r="C95" s="4"/>
       <c r="D95" s="4"/>
@@ -11133,7 +11188,7 @@
       <c r="K95" s="4"/>
       <c r="L95" s="4"/>
     </row>
-    <row r="96" spans="2:12">
+    <row r="96" spans="1:12">
       <c r="B96" s="4"/>
       <c r="C96" s="4"/>
       <c r="D96" s="4"/>

</xml_diff>

<commit_message>
updated the new files
</commit_message>
<xml_diff>
--- a/Project_Roadmap_Ashwini.xlsx
+++ b/Project_Roadmap_Ashwini.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\E drive\Previous data\Project\52 project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80FF80C3-60EA-4217-8E88-1947421DF20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10A95F89-A6A4-42D6-96F1-87D9240EA0A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12960" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12960" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -10565,7 +10565,7 @@
       <c r="B65" s="1">
         <v>60</v>
       </c>
-      <c r="C65" s="1" t="s">
+      <c r="C65" s="13" t="s">
         <v>134</v>
       </c>
       <c r="D65" s="1" t="s">

</xml_diff>